<commit_message>
Regelkatalog 0.15.0: 82/163 (4 beregningsregler) + governance-pakke regenereret
</commit_message>
<xml_diff>
--- a/docs/Pillar2-Validator_Regel-sporbarhedsmatrix.xlsx
+++ b/docs/Pillar2-Validator_Regel-sporbarhedsmatrix.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3020,7 +3020,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>70088</t>
+          <t>70087</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3030,17 +3030,17 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Negativ NetGlobeIncome kræver Art4.1.5</t>
+          <t>SubstanceExclusion/Total-beregning</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70088</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70087</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -3062,7 +3062,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>70090</t>
+          <t>70088</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3072,17 +3072,17 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>GlobeLoss skal svare til NetGlobeIncome/Total</t>
+          <t>Negativ NetGlobeIncome kræver Art4.1.5</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70090</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70088</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -3104,7 +3104,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>70093</t>
+          <t>70090</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3114,17 +3114,17 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>NONArt4.1.5-år må ikke overstige periodens slut</t>
+          <t>GlobeLoss skal svare til NetGlobeIncome/Total</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70093</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70090</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>70101</t>
+          <t>70091</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -3156,17 +3156,17 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Employees kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
+          <t>ExpectedAdjustedCoveredTax = GlobeLoss × 15%</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70101</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70091</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -3188,7 +3188,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>70102</t>
+          <t>70093</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3198,17 +3198,17 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>TangibleAssetValue kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
+          <t>NONArt4.1.5-år må ikke overstige periodens slut</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70102</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70093</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -3230,7 +3230,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>70103</t>
+          <t>70097</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3240,17 +3240,17 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>UTPRPercentage skal være 0 når carryforward &gt; 0</t>
+          <t>InclusionRatio-beregning</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70103</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70097</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -3272,7 +3272,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>70104</t>
+          <t>70098</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3282,17 +3282,17 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>value_range</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>UTPRTopUpTaxCarriedForward må ikke være negativ</t>
+          <t>TopUpTaxShare = TopUpTax × InclusionRatio</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70104</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70098</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -3314,7 +3314,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>70105</t>
+          <t>70101</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3324,17 +3324,17 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>UTPRTopUpTaxCarriedForward-beregning</t>
+          <t>Employees kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70105</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70101</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -3356,7 +3356,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>70107</t>
+          <t>70102</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3371,12 +3371,12 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Exception=TRUE udelukker CrossBorderAdjustments</t>
+          <t>TangibleAssetValue kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70107</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70102</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -3398,7 +3398,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>70108</t>
+          <t>70103</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -3413,12 +3413,12 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Basis kræver TaxRate</t>
+          <t>UTPRPercentage skal være 0 når carryforward &gt; 0</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70108</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70103</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -3440,7 +3440,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>70109</t>
+          <t>70104</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3450,17 +3450,17 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>value_range</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1907 kræver IndOwners/ResCountryCode</t>
+          <t>UTPRTopUpTaxCarriedForward må ikke være negativ</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70109</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70104</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -3482,7 +3482,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>70110</t>
+          <t>70105</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3492,17 +3492,17 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1903/1908 kræver IndOwners</t>
+          <t>UTPRTopUpTaxCarriedForward-beregning</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70110</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70105</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -3524,7 +3524,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>70111</t>
+          <t>70107</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3539,12 +3539,12 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1904/1909 kræver EntityOwner/ExTypeOfEntity</t>
+          <t>Exception=TRUE udelukker CrossBorderAdjustments</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70111</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70107</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -3566,7 +3566,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>70112</t>
+          <t>70108</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -3581,12 +3581,12 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1904 udelukker ExTypeOfEntity GIR2805</t>
+          <t>Basis kræver TaxRate</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70112</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70108</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -3608,7 +3608,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>70113</t>
+          <t>70109</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -3623,12 +3623,12 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1909 udelukker ExTypeOfEntity GIR2804</t>
+          <t>Basis GIR1907 kræver IndOwners/ResCountryCode</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70113</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70109</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -3650,7 +3650,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>70115</t>
+          <t>70110</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -3665,12 +3665,12 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem GIR2022/2023 kræver UPEAdjustments</t>
+          <t>Basis GIR1903/1908 kræver IndOwners</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70115</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70110</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -3692,7 +3692,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>70123</t>
+          <t>70111</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3702,17 +3702,17 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>value_range</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Additions må ikke være negativ</t>
+          <t>Basis GIR1904/1909 kræver EntityOwner/ExTypeOfEntity</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70123</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70111</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -3734,40 +3734,208 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
+          <t>70112</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Basis GIR1904 udelukker ExTypeOfEntity GIR2805</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70112</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>70113</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Basis GIR1909 udelukker ExTypeOfEntity GIR2804</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70113</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>70115</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>AdjustmentItem GIR2022/2023 kræver UPEAdjustments</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70115</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>70123</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>value_range</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Additions må ikke være negativ</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70123</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
           <t>70124</t>
         </is>
       </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
         <is>
           <t>value_range</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
+      <c r="D83" s="2" t="inlineStr">
         <is>
           <t>CrossAllocation/Reductions må ikke være positiv</t>
         </is>
       </c>
-      <c r="E79" s="2" t="inlineStr">
+      <c r="E83" s="2" t="inlineStr">
         <is>
           <t>OECD Status Message User Guide Part 4 — regel 70124</t>
         </is>
       </c>
-      <c r="F79" s="2" t="inlineStr">
+      <c r="F83" s="2" t="inlineStr">
         <is>
           <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
         </is>
       </c>
-      <c r="G79" s="2" t="inlineStr">
+      <c r="G83" s="2" t="inlineStr">
         <is>
           <t>Ja — auto-scenarie (bestået)</t>
         </is>
       </c>
-      <c r="H79" s="2" t="inlineStr">
+      <c r="H83" s="2" t="inlineStr">
         <is>
           <t>Væsentlig (High)</t>
         </is>
@@ -8205,7 +8373,7 @@
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -8349,7 +8517,7 @@
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
@@ -8571,7 +8739,7 @@
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
@@ -8608,7 +8776,7 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Regelkatalog 0.16.0: dato-aware conditional (ref/offset) + 5 regler (87/163) + pakke regenereret
</commit_message>
<xml_diff>
--- a/docs/Pillar2-Validator_Regel-sporbarhedsmatrix.xlsx
+++ b/docs/Pillar2-Validator_Regel-sporbarhedsmatrix.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1928,7 +1928,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>70044</t>
+          <t>70038</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1943,12 +1943,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>ETRStatus skal indeholde ETRException eller ETRComputation</t>
+          <t>Transitional CbCR SafeHarbour udløber efter 30/06/2028</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70044</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70038</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1970,7 +1970,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>70045</t>
+          <t>70039</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1985,12 +1985,12 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1203-1205 kræver TransitionalCbCRSafeHarbour</t>
+          <t>UTPR SafeHarbour (GIR1206) udløber efter 31/12/2026</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70045</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70039</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2012,7 +2012,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>70047</t>
+          <t>70044</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2027,12 +2027,12 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1203 kræver Revenue</t>
+          <t>ETRStatus skal indeholde ETRException eller ETRComputation</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70047</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70044</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2054,7 +2054,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>70048</t>
+          <t>70045</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2069,12 +2069,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1204 kræver IncomeTax</t>
+          <t>SafeHarbour GIR1203-1205 kræver TransitionalCbCRSafeHarbour</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70048</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70045</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2096,7 +2096,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>70049</t>
+          <t>70047</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2111,12 +2111,12 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1206 kræver UTPRSafeHarbour</t>
+          <t>SafeHarbour GIR1203 kræver Revenue</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70049</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70047</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2138,7 +2138,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>70051</t>
+          <t>70048</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2153,12 +2153,12 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1208 kræver AggregateSimplified</t>
+          <t>SafeHarbour GIR1204 kræver IncomeTax</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70051</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70048</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2180,7 +2180,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>70055</t>
+          <t>70049</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2190,17 +2190,17 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>OutstandingBalance-beregning</t>
+          <t>SafeHarbour GIR1206 kræver UTPRSafeHarbour</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70055</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70049</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2222,7 +2222,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>70059</t>
+          <t>70051</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2232,17 +2232,17 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>unique_in</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem-kode kun én gang pr. ETR</t>
+          <t>SafeHarbour GIR1208 kræver AggregateSimplified</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70059</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70051</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2264,7 +2264,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>70060</t>
+          <t>70055</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2274,17 +2274,17 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem GIR2025 kræver IntShippingIncome</t>
+          <t>OutstandingBalance-beregning</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70060</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70055</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>70062</t>
+          <t>70059</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2316,17 +2316,17 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>unique_in</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem GIR2720 udelukker negativ AdjustedCoveredTax</t>
+          <t>AdjustmentItem-kode kun én gang pr. ETR</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70062</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70059</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2348,7 +2348,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>70064</t>
+          <t>70060</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2358,17 +2358,17 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>DeferTaxAsset/Total-beregning</t>
+          <t>AdjustmentItem GIR2025 kræver IntShippingIncome</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70064</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70060</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2390,7 +2390,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>70065</t>
+          <t>70062</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2400,17 +2400,17 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>CoveredTaxRefund/Total-beregning</t>
+          <t>AdjustmentItem GIR2720 udelukker negativ AdjustedCoveredTax</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70065</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70062</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2432,7 +2432,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>70066</t>
+          <t>70064</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2442,17 +2442,17 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>DeferTaxAsset-år må ikke ligge efter periodens start</t>
+          <t>DeferTaxAsset/Total-beregning</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70066</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70064</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2474,7 +2474,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>70067</t>
+          <t>70065</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2484,17 +2484,17 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>unique_in</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>AmountAttributed-år skal være unikke</t>
+          <t>CoveredTaxRefund/Total-beregning</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70067</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70065</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2516,7 +2516,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>70068</t>
+          <t>70066</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2531,12 +2531,12 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>CoveredTaxRefund-år må ikke ligge efter periodens start</t>
+          <t>DeferTaxAsset-år må ikke ligge efter periodens start</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70068</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70066</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2558,7 +2558,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>70070</t>
+          <t>70067</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2568,17 +2568,17 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>unique_in</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Recapture-år må ikke ligge efter periodens slut</t>
+          <t>AmountAttributed-år skal være unikke</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70070</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70067</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2600,7 +2600,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>70072</t>
+          <t>70068</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2610,17 +2610,17 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>EndAmount-beregning (DDT-recapture)</t>
+          <t>CoveredTaxRefund-år må ikke ligge efter periodens start</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70072</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70068</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2642,7 +2642,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>70073</t>
+          <t>70070</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2652,17 +2652,17 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>value_range</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>EndAmount må ikke være negativ</t>
+          <t>Recapture-år må ikke ligge efter periodens slut</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70073</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70070</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2684,7 +2684,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>70074</t>
+          <t>70071</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>TotalDDT-beregning</t>
+          <t>Recapture-år må ikke være 4+ år før periodens slut</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70074</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70071</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2726,7 +2726,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>70076</t>
+          <t>70072</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2741,12 +2741,12 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>TransBlendCFC/Total-beregning</t>
+          <t>EndAmount-beregning (DDT-recapture)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70076</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70072</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -2768,7 +2768,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>70077</t>
+          <t>70073</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2778,17 +2778,17 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>value_range</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>DeferTaxAdjustAmt/Total-beregning (Recast)</t>
+          <t>EndAmount må ikke være negativ</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70077</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70073</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2810,7 +2810,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>70078</t>
+          <t>70074</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2825,12 +2825,12 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>BefRecastAdjust-beregning</t>
+          <t>TotalDDT-beregning</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70078</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70074</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2852,7 +2852,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>70079</t>
+          <t>70076</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2867,12 +2867,12 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>PreRecast-beregning</t>
+          <t>TransBlendCFC/Total-beregning</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70079</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70076</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -2894,7 +2894,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>70082</t>
+          <t>70077</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2904,17 +2904,17 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>DeferredTaxAssets kræver Start eller Recast = 0</t>
+          <t>DeferTaxAdjustAmt/Total-beregning (Recast)</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70082</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70077</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -2936,7 +2936,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>70083</t>
+          <t>70078</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2951,12 +2951,12 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>ExcessNegTaxExpense/Remaining-beregning</t>
+          <t>BefRecastAdjust-beregning</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70083</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70078</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -2978,7 +2978,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>70086</t>
+          <t>70079</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2993,12 +2993,12 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>ExcessProfits-beregning</t>
+          <t>PreRecast-beregning</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70086</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70079</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -3020,7 +3020,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>70087</t>
+          <t>70082</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3030,17 +3030,17 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>SubstanceExclusion/Total-beregning</t>
+          <t>DeferredTaxAssets kræver Start eller Recast = 0</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70087</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70082</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -3062,7 +3062,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>70088</t>
+          <t>70083</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3072,17 +3072,17 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Negativ NetGlobeIncome kræver Art4.1.5</t>
+          <t>ExcessNegTaxExpense/Remaining-beregning</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70088</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70083</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -3104,7 +3104,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>70090</t>
+          <t>70086</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3119,12 +3119,12 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>GlobeLoss skal svare til NetGlobeIncome/Total</t>
+          <t>ExcessProfits-beregning</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70090</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70086</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>70091</t>
+          <t>70087</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -3161,12 +3161,12 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>ExpectedAdjustedCoveredTax = GlobeLoss × 15%</t>
+          <t>SubstanceExclusion/Total-beregning</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70091</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70087</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -3188,7 +3188,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>70093</t>
+          <t>70088</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3198,17 +3198,17 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>NONArt4.1.5-år må ikke overstige periodens slut</t>
+          <t>Negativ NetGlobeIncome kræver Art4.1.5</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70093</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70088</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -3230,7 +3230,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>70097</t>
+          <t>70090</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3245,12 +3245,12 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>InclusionRatio-beregning</t>
+          <t>GlobeLoss skal svare til NetGlobeIncome/Total</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70097</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70090</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -3272,7 +3272,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>70098</t>
+          <t>70091</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3287,12 +3287,12 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>TopUpTaxShare = TopUpTax × InclusionRatio</t>
+          <t>ExpectedAdjustedCoveredTax = GlobeLoss × 15%</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70098</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70091</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -3314,7 +3314,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>70101</t>
+          <t>70093</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3324,17 +3324,17 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Employees kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
+          <t>NONArt4.1.5-år må ikke overstige periodens slut</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70101</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70093</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -3356,7 +3356,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>70102</t>
+          <t>70094</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3371,12 +3371,12 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>TangibleAssetValue kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
+          <t>Articles GIR2605 kræver år mindst 4 år før periodens slut</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70102</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70094</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -3398,7 +3398,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>70103</t>
+          <t>70095</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -3413,12 +3413,12 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>UTPRPercentage skal være 0 når carryforward &gt; 0</t>
+          <t>Articles GIR2602 kræver det femte år før periodens slut</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70103</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70095</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -3440,7 +3440,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>70104</t>
+          <t>70097</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3450,17 +3450,17 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>value_range</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>UTPRTopUpTaxCarriedForward må ikke være negativ</t>
+          <t>InclusionRatio-beregning</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70104</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70097</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -3482,7 +3482,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>70105</t>
+          <t>70098</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3497,12 +3497,12 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>UTPRTopUpTaxCarriedForward-beregning</t>
+          <t>TopUpTaxShare = TopUpTax × InclusionRatio</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70105</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70098</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -3524,7 +3524,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>70107</t>
+          <t>70101</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3539,12 +3539,12 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Exception=TRUE udelukker CrossBorderAdjustments</t>
+          <t>Employees kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70107</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70101</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -3566,7 +3566,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>70108</t>
+          <t>70102</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -3581,12 +3581,12 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Basis kræver TaxRate</t>
+          <t>TangibleAssetValue kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70108</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70102</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -3608,7 +3608,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>70109</t>
+          <t>70103</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -3623,12 +3623,12 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1907 kræver IndOwners/ResCountryCode</t>
+          <t>UTPRPercentage skal være 0 når carryforward &gt; 0</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70109</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70103</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -3650,7 +3650,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>70110</t>
+          <t>70104</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -3660,17 +3660,17 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>value_range</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1903/1908 kræver IndOwners</t>
+          <t>UTPRTopUpTaxCarriedForward må ikke være negativ</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70110</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70104</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -3692,7 +3692,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>70111</t>
+          <t>70105</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3702,17 +3702,17 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1904/1909 kræver EntityOwner/ExTypeOfEntity</t>
+          <t>UTPRTopUpTaxCarriedForward-beregning</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70111</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70105</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -3734,7 +3734,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>70112</t>
+          <t>70107</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -3749,12 +3749,12 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1904 udelukker ExTypeOfEntity GIR2805</t>
+          <t>Exception=TRUE udelukker CrossBorderAdjustments</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70112</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70107</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -3776,7 +3776,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>70113</t>
+          <t>70108</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -3791,12 +3791,12 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1909 udelukker ExTypeOfEntity GIR2804</t>
+          <t>Basis kræver TaxRate</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70113</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70108</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -3818,7 +3818,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>70115</t>
+          <t>70109</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -3833,12 +3833,12 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem GIR2022/2023 kræver UPEAdjustments</t>
+          <t>Basis GIR1907 kræver IndOwners/ResCountryCode</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70115</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70109</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -3860,7 +3860,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>70123</t>
+          <t>70110</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -3870,17 +3870,17 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>value_range</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Additions må ikke være negativ</t>
+          <t>Basis GIR1903/1908 kræver IndOwners</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70123</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70110</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -3902,40 +3902,250 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
+          <t>70111</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Basis GIR1904/1909 kræver EntityOwner/ExTypeOfEntity</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70111</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>70112</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Basis GIR1904 udelukker ExTypeOfEntity GIR2805</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70112</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>70113</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Basis GIR1909 udelukker ExTypeOfEntity GIR2804</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70113</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>70115</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>AdjustmentItem GIR2022/2023 kræver UPEAdjustments</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70115</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>70123</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>value_range</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Additions må ikke være negativ</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70123</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
           <t>70124</t>
         </is>
       </c>
-      <c r="B83" s="2" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="C83" s="2" t="inlineStr">
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t>value_range</t>
         </is>
       </c>
-      <c r="D83" s="2" t="inlineStr">
+      <c r="D88" s="2" t="inlineStr">
         <is>
           <t>CrossAllocation/Reductions må ikke være positiv</t>
         </is>
       </c>
-      <c r="E83" s="2" t="inlineStr">
+      <c r="E88" s="2" t="inlineStr">
         <is>
           <t>OECD Status Message User Guide Part 4 — regel 70124</t>
         </is>
       </c>
-      <c r="F83" s="2" t="inlineStr">
+      <c r="F88" s="2" t="inlineStr">
         <is>
           <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
         </is>
       </c>
-      <c r="G83" s="2" t="inlineStr">
+      <c r="G88" s="2" t="inlineStr">
         <is>
           <t>Ja — auto-scenarie (bestået)</t>
         </is>
       </c>
-      <c r="H83" s="2" t="inlineStr">
+      <c r="H88" s="2" t="inlineStr">
         <is>
           <t>Væsentlig (High)</t>
         </is>
@@ -6600,7 +6810,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -6637,7 +6847,7 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -7793,7 +8003,7 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
@@ -8628,7 +8838,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -8665,7 +8875,7 @@
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Regel-triage 0.17.0: ærligt dækningsbillede (scope-klassifikation, 92/143 fil-validerbare) + docx selvberegnende
</commit_message>
<xml_diff>
--- a/docs/Pillar2-Validator_Regel-sporbarhedsmatrix.xlsx
+++ b/docs/Pillar2-Validator_Regel-sporbarhedsmatrix.xlsx
@@ -7,16 +7,18 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sporbarhed" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuldt katalog" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referencedata" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Severity &amp; materialitet" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dækningsoverblik" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sporbarhed" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuldt katalog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referencedata" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Severity &amp; materialitet" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sporbarhed'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fuldt katalog'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Referencedata'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Severity &amp; materialitet'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dækningsoverblik'!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sporbarhed'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fuldt katalog'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Referencedata'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Severity &amp; materialitet'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,6 +444,172 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Antal</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Forklaring</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Eksekverbare kontroller</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Kodet i regelmotoren og verificeret af valideringssuiten (én planted defekt pr. kontrol).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Dækket af ækvivalent regel</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Samme semantik håndhæves allerede af en eksekverbar regel (fx AdjustmentItem-unikhed pr. ETR).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Kandidater (kan kodes)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Fil-validerbare regler der endnu ikke er kodet; kodes batch-vis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Uden for scope (fil-validering)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Transmissions-/modtagerstatus, kryds-besked-/korrektionshistorik eller eksternt register — kan ikke afgøres ud fra én GIR-fils indhold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Slået fra (2026-guidance)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Fyres aldrig jf. juni-2026-guidance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>I ALT (officielt katalog)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>163</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Fil-validerbare regler i alt</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>143</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Officielt katalog minus switched-off og uden-for-scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Effektivt dækket</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Eksekverbare + dækket-af-ækvivalent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Dækningsgrad (fil-validerbare)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>64%</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4157,7 +4325,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4168,11 +4336,11 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4193,12 +4361,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Eksekverbar</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Switched-off 2026</t>
+          <t>Begrundelse / dækket af</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -4230,12 +4398,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Transmissions-/modtagerstatus — genereres af den modtagende myndighed (download, dekryptering, dekomprimering, signatur, sikkerhed/virus); kan ikke afgøres ud fra en GIR-fils indhold.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
@@ -4259,12 +4427,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Transmissions-/modtagerstatus — genereres af den modtagende myndighed (download, dekryptering, dekomprimering, signatur, sikkerhed/virus); kan ikke afgøres ud fra en GIR-fils indhold.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -4288,12 +4456,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Transmissions-/modtagerstatus — genereres af den modtagende myndighed (download, dekryptering, dekomprimering, signatur, sikkerhed/virus); kan ikke afgøres ud fra en GIR-fils indhold.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
@@ -4317,12 +4485,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Transmissions-/modtagerstatus — genereres af den modtagende myndighed (download, dekryptering, dekomprimering, signatur, sikkerhed/virus); kan ikke afgøres ud fra en GIR-fils indhold.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
@@ -4346,12 +4514,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Transmissions-/modtagerstatus — genereres af den modtagende myndighed (download, dekryptering, dekomprimering, signatur, sikkerhed/virus); kan ikke afgøres ud fra en GIR-fils indhold.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
@@ -4375,12 +4543,12 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Transmissions-/modtagerstatus — genereres af den modtagende myndighed (download, dekryptering, dekomprimering, signatur, sikkerhed/virus); kan ikke afgøres ud fra en GIR-fils indhold.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
@@ -4404,12 +4572,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Status-kode for skemavalidering hos modtager — substansen dækkes allerede af lag 1 (XSD-validering, P2-001).</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
@@ -4433,12 +4601,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Transmissions-/modtagerstatus — genereres af den modtagende myndighed (download, dekryptering, dekomprimering, signatur, sikkerhed/virus); kan ikke afgøres ud fra en GIR-fils indhold.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -4466,12 +4634,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Transmissions-/modtagerstatus — genereres af den modtagende myndighed (download, dekryptering, dekomprimering, signatur, sikkerhed/virus); kan ikke afgøres ud fra en GIR-fils indhold.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -4499,12 +4667,12 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Transmissions-/modtagerstatus — genereres af den modtagende myndighed (download, dekryptering, dekomprimering, signatur, sikkerhed/virus); kan ikke afgøres ud fra en GIR-fils indhold.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -4532,12 +4700,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Transmissions-/modtagerstatus — genereres af den modtagende myndighed (download, dekryptering, dekomprimering, signatur, sikkerhed/virus); kan ikke afgøres ud fra en GIR-fils indhold.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
@@ -4561,14 +4729,10 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
           <t>MessageSpec/MessageRefId</t>
@@ -4594,12 +4758,12 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Dublet-MessageRefId modtaget på en TIDLIGERE fil — kræver beskedhistorik på tværs af filer.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -4627,14 +4791,10 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>MessageSpec/ReportingPeriod</t>
@@ -4660,14 +4820,10 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
           <t>.//DocTypeIndic</t>
@@ -4693,14 +4849,10 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
           <t>.//DocTypeIndic</t>
@@ -4726,14 +4878,10 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
           <t>.//CorrDocRefID</t>
@@ -4759,14 +4907,10 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
           <t>.//DocRefId</t>
@@ -4792,12 +4936,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>CorrDocRefId henviser til en ukendt post — kræver postregister/historik fra tidligere indsendelser.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -4825,12 +4969,12 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>CorrDocRefId skal pege på seneste instans af DocRefId — kræver korrektionshistorik på tværs af beskeder.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -4858,14 +5002,10 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/FilingInfo/DocSpec/DocTypeIndic</t>
@@ -4891,14 +5031,10 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
           <t>.//DocRefId</t>
@@ -4924,14 +5060,10 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
           <t>.//CorrDocRefId</t>
@@ -4957,14 +5089,10 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/DocSpec/DocTypeIndicGLOBEBody/Summary/DocSpec/DocTypeIndicGLOBEBody/JurisdictionSection/DocSpec/DocTypeIndicGLOBEBody/UTPRAttribution/DocSpec/DocTypeIndic</t>
@@ -4990,12 +5118,12 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>OECD0/resend: DocRefID skal matche en tidligere brugt DocRefID — kræver beskedhistorik.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -5023,14 +5151,10 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr">
         <is>
           <t>.//CorrDocRefId</t>
@@ -5056,14 +5180,10 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
           <t>GloBEBody/FilingInfo/DocSpec/DocTypeIndicGloBEBody/GeneralSection/DocSpec/DocTypeIndic</t>
@@ -5089,14 +5209,10 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
           <t>GloBEBody/FilingInfo/DocSpec/DocTypeIndicGloBEBody/GeneralSection</t>
@@ -5122,14 +5238,10 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
           <t>.//RecJurCode</t>
@@ -5155,14 +5267,10 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
           <t>.//RecJurCode</t>
@@ -5188,14 +5296,10 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/FilingInfo/Period/Start</t>
@@ -5225,14 +5329,10 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/FilingInfo/Period/End</t>
@@ -5262,14 +5362,10 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/FilingInfo/FilingCE/TIN</t>
@@ -5299,14 +5395,10 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/FilingInfo/FilingCE/ResCountryCode</t>
@@ -5336,14 +5428,10 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/Summary/JurWithTaxingRights</t>
@@ -5373,14 +5461,10 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Ja (fyres aldrig)</t>
-        </is>
-      </c>
+          <t>Slået fra (2026-guidance)</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/ETRRate</t>
@@ -5410,14 +5494,10 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Ja (fyres aldrig)</t>
-        </is>
-      </c>
+          <t>Slået fra (2026-guidance)</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/TopUpTax</t>
@@ -5447,14 +5527,10 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/LowTaxJurisdiction/LTCE/IIR/ParentEntity/TopUpTax</t>
@@ -5484,14 +5560,10 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedFANIL/Total</t>
@@ -5521,14 +5593,10 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="2" t="inlineStr">
         <is>
           <t>.//TIN</t>
@@ -5554,14 +5622,10 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr">
         <is>
           <t>.//TIN</t>
@@ -5587,14 +5651,10 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr"/>
       <c r="F43" s="2" t="inlineStr">
         <is>
           <t>.//TIN</t>
@@ -5620,12 +5680,12 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Uden for scope (fil-validering)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>TIN skal være en gyldig TIN i den lokale jurisdiktion — kræver eksternt TIN-register.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -5653,14 +5713,10 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr">
         <is>
           <t>.//TIN</t>
@@ -5686,14 +5742,10 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/UPE/ExcludedUPE/ID/TINGLOBEBody/GeneralSection/CorporateStructure/UPE/OtherUPE/ID/TINGLOBEBody/GeneralSection/CorporateStructure/CE/ID/TINGLOBEBody/GeneralSection/CorporateStructure/CE/QIIR/Exception/TINGLOBEBody/GeneralSection/CorporateStructure/CE/ID/TINGLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/CEComputation/Elections/AggregatedReporting/TaxConsolGroupTIN</t>
@@ -5719,14 +5771,10 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
           <t>.//TIN</t>
@@ -5752,14 +5800,10 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
           <t>GloBEBody/UTPRAttribution/RecJurCode</t>
@@ -5789,14 +5833,10 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr"/>
       <c r="F49" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/UPE/ExcludedUPE/ID/GloBEStatusGLOBEBody/GeneralSection/CorporateStructure/UPE/OtherUPE/ID/GloBEStatus</t>
@@ -5822,14 +5862,10 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr"/>
       <c r="F50" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/UPE/OtherUPE/ID/ResCountryCode</t>
@@ -5855,14 +5891,10 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr"/>
       <c r="F51" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/ID/ResCountryCode</t>
@@ -5888,14 +5920,10 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/UPE/ExcludedUPE/ID/RulesGLOBEBody/GeneralSection/CorporateStructure/UPE/OtherUPE/ID/RulesGLOBEBody/GeneralSection/CorporateStructure/CE/ID/Rules</t>
@@ -5921,14 +5949,10 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/ID/GloBEStatus</t>
@@ -5954,14 +5978,10 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/ID/GloBEStatus</t>
@@ -5987,14 +6007,10 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr"/>
       <c r="F55" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/ID/GloBEStatus</t>
@@ -6020,14 +6036,10 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr"/>
       <c r="F56" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/ID/GloBEStatus</t>
@@ -6053,14 +6065,10 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
       <c r="F57" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/ID/GloBEStatus</t>
@@ -6086,14 +6094,10 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr"/>
       <c r="F58" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/ID/GloBEStatus</t>
@@ -6119,14 +6123,10 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr"/>
       <c r="F59" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/ID/GloBEStatus</t>
@@ -6152,14 +6152,10 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
       <c r="F60" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/ID/GloBEStatus</t>
@@ -6185,14 +6181,10 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr"/>
       <c r="F61" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/ID/GloBEStatus</t>
@@ -6222,14 +6214,10 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr"/>
       <c r="F62" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/OwnershipChange/ChangeDate</t>
@@ -6259,14 +6247,10 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr"/>
       <c r="F63" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/OwnershipChange/ChangeDate</t>
@@ -6296,14 +6280,10 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr"/>
       <c r="F64" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/OwnershipChange/PreOwnership</t>
@@ -6333,14 +6313,10 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr"/>
       <c r="F65" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/OwnershipChange/PreOwnership/TIN</t>
@@ -6370,14 +6346,10 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/Ownership/OwnershipPercentage</t>
@@ -6407,14 +6379,10 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr"/>
       <c r="F67" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/Ownership/OwnershipPercentageGLOBEBody/GeneralSection/CorporateStructure/CE/Ownership/TINGLOBEBody/GeneralSection/CorporateStructure/CE/Ownership/OwnershipType</t>
@@ -6444,14 +6412,10 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>Ja (fyres aldrig)</t>
-        </is>
-      </c>
+          <t>Slået fra (2026-guidance)</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/Ownership/OwnershipPercentage</t>
@@ -6481,14 +6445,10 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr"/>
       <c r="F69" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/Ownership/TIN</t>
@@ -6518,14 +6478,10 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr"/>
       <c r="F70" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/Ownership/TIN</t>
@@ -6555,14 +6511,10 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr"/>
       <c r="F71" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/Ownership/TIN</t>
@@ -6592,14 +6544,10 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr"/>
       <c r="F72" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/QIIR</t>
@@ -6629,14 +6577,10 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr"/>
       <c r="F73" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/QIIR/Exception/TIN</t>
@@ -6666,14 +6610,10 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr"/>
       <c r="F74" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/QIIR/Exception/Art2.1.3</t>
@@ -6703,14 +6643,10 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr"/>
       <c r="F75" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/GeneralSection/CorporateStructure/CE/QIIR/Exception/Art2.1.5</t>
@@ -6740,14 +6676,10 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/Summary/Jurisdiction/Subgroup</t>
@@ -6773,14 +6705,10 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/Subgroup/TIN</t>
@@ -6810,14 +6738,10 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr"/>
       <c r="F78" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/Summary/SafeHarbour</t>
@@ -6847,14 +6771,10 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr"/>
       <c r="F79" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/Summary/SafeHarbour</t>
@@ -6884,14 +6804,10 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/Summary/SafeHarbour</t>
@@ -6921,14 +6837,10 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr"/>
       <c r="F81" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/Summary/SafeHarbour</t>
@@ -6958,14 +6870,10 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr"/>
       <c r="F82" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/Summary/ETRRangeGLOBEBody/Summary/SBIEGLOBEBody/Summary/QDMTTutGLOBEBody/Summary/GloBETut</t>
@@ -6995,14 +6903,10 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E83" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr"/>
       <c r="F83" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/Summary/ETRRangeGLOBEBody/Summary/SBIEGLOBEBody/Summary/QDMTTut</t>
@@ -7032,14 +6936,10 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr"/>
       <c r="F84" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus</t>
@@ -7065,14 +6965,10 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr"/>
       <c r="F85" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRException/TransitionalCbCRSafeHarbour</t>
@@ -7102,14 +6998,10 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/SubGroupGLOBEBody/JurisdictionSection/GLoBETax/ETR/SubGroup/TypeofSubGroup</t>
@@ -7139,14 +7031,10 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr"/>
       <c r="F87" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/Summary/SafeHarbour</t>
@@ -7176,14 +7064,10 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr"/>
       <c r="F88" s="2" t="inlineStr">
         <is>
           <t>GLOEBody/Summary/SafeHarbour</t>
@@ -7213,14 +7097,10 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr"/>
       <c r="F89" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/Summary/SafeHarbour</t>
@@ -7250,14 +7130,10 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr"/>
       <c r="F90" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/Summary/SafeHarbour</t>
@@ -7287,14 +7163,10 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr"/>
       <c r="F91" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/Summary/SafeHarbour</t>
@@ -7324,14 +7196,10 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr"/>
       <c r="F92" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETAX/ETR/ETRStatus/ETRComputation/OverallComputation/SubstanceExclusionSummary/SafeHarbourJurisdictionSection/GLOBETAX/ETR/ETRStatus/ETRComputation/OverallComputation/SubstanceExclusion</t>
@@ -7357,14 +7225,10 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E93" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr"/>
       <c r="F93" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETAX/ETR/ETRStatus/ETRComputation/OverallComputation/SubstanceExclusionSummary/SafeHarbourJurisdictionSection/GLOBETAX/ETR/ETRStatus/ETRComputation/OverallComputation/SubstanceExclusionJurisdictionSection/GLoBETax/ETR/ETRStatus/ETRException/TransitionalCbCRSafeHarbour/Profit</t>
@@ -7390,14 +7254,10 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E94" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr"/>
       <c r="F94" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/Election/*/RevocationYear</t>
@@ -7427,14 +7287,10 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E95" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr"/>
       <c r="F95" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/Election/Art3.2.1.c/OutstandingBalance</t>
@@ -7464,14 +7320,10 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E96" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr"/>
       <c r="F96" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/Elections/*/RevocationYear</t>
@@ -7501,14 +7353,10 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E97" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr"/>
       <c r="F97" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/TIN</t>
@@ -7538,14 +7386,10 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E98" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr"/>
       <c r="F98" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/Elections/Art7.6/InvestmentEntityTIN</t>
@@ -7575,14 +7419,10 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E99" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr"/>
       <c r="F99" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/NetGlobeIncome/Adjustments/AdjustmentItem</t>
@@ -7608,14 +7448,10 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr"/>
       <c r="F100" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/NetGlobeIncome/IntShippingIncome</t>
@@ -7645,14 +7481,10 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr"/>
       <c r="F101" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/Adjustments/AdjustmentItemGLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/Adjustments/Amount</t>
@@ -7682,14 +7514,10 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E102" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr"/>
       <c r="F102" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/Total</t>
@@ -7719,12 +7547,12 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Dækket af ækvivalent regel</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Samme semantik håndhæves allerede af regel 70059.</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -7752,14 +7580,10 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr"/>
       <c r="F104" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/PostFilingAdjust/DeferTaxAsset/Total</t>
@@ -7789,14 +7613,10 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr"/>
       <c r="F105" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/PostFilingAdjust/CoveredTaxRefund/Total</t>
@@ -7826,14 +7646,10 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E106" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr"/>
       <c r="F106" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/PostFilingAdjust/DeferTaxAsset/AmountAttributed/Year</t>
@@ -7863,14 +7679,10 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E107" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr"/>
       <c r="F107" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/PostFilingAdjust/DeferTaxAsset/AmountAttributed/Year</t>
@@ -7896,14 +7708,10 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E108" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr"/>
       <c r="F108" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/PostFilingAdjust/CoveredTaxRefund/AmountAttributed/Year</t>
@@ -7933,12 +7741,12 @@
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Dækket af ækvivalent regel</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Samme semantik håndhæves allerede af regel 70067.</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
@@ -7966,14 +7774,10 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr"/>
       <c r="F110" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeemedDistTax/Election/Recapture/Year</t>
@@ -8003,14 +7807,10 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E111" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr"/>
       <c r="F111" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeemedDistTax/Election/Recapture/Year</t>
@@ -8040,14 +7840,10 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E112" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr"/>
       <c r="F112" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeemedDistTax/Election/Recapture/EndAmount</t>
@@ -8077,14 +7873,10 @@
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E113" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr"/>
       <c r="F113" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeemedDistTax/Election/Recapture/EndAmount</t>
@@ -8110,14 +7902,10 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E114" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr"/>
       <c r="F114" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeemedDistTax/Election/Recapture/TotalDDT</t>
@@ -8147,14 +7935,10 @@
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E115" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr"/>
       <c r="F115" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeemedDistTax/Election/Recapture/DDTYear-0GLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeemedDistTax/Election/Recapture/DDTYear-1GLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeemedDistTax/Election/Recapture/DDTYear-2GLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeemedDistTax/Election/Recapture/DDTYear-3</t>
@@ -8184,14 +7968,10 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E116" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr"/>
       <c r="F116" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/TransBlendCFC/Total</t>
@@ -8221,14 +8001,10 @@
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E117" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr"/>
       <c r="F117" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeferTaxAdjustAmt/Total</t>
@@ -8254,14 +8030,10 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E118" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr"/>
       <c r="F118" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeferTaxAdjustAmt/BefRecastAdjust</t>
@@ -8291,14 +8063,10 @@
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E119" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr"/>
       <c r="F119" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeferTaxAdjustAmt/PreRecast</t>
@@ -8328,12 +8096,12 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Dækket af ækvivalent regel</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Samme semantik håndhæves allerede af regel 70059.</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
@@ -8361,14 +8129,10 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E121" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr"/>
       <c r="F121" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeferTaxAdjustAmt/Transition/DeferredTaxAssets/Total</t>
@@ -8398,14 +8162,10 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E122" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr"/>
       <c r="F122" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeferTaxAdjustAmt/Transition/DeferredTaxAssets/DeferredTaxAssetStartGLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/DeferTaxAdjustAmt/Transition/DeferredTaxAssets/DeferredTaxAssetRecast</t>
@@ -8435,14 +8195,10 @@
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E123" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr"/>
       <c r="F123" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/ExcessNegTaxExpense/Remaining</t>
@@ -8472,14 +8228,10 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E124" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr"/>
       <c r="F124" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/Adjustments/Amount</t>
@@ -8509,14 +8261,10 @@
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E125" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr"/>
       <c r="F125" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdjustedCoveredTax/Adjustments/Amount</t>
@@ -8546,14 +8294,10 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E126" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr"/>
       <c r="F126" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/ExcessProfits</t>
@@ -8583,14 +8327,10 @@
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E127" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr"/>
       <c r="F127" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETAX/ETR/ETRStatus/ETRComputation/OverallComputation/SubstanceExclusion/Total</t>
@@ -8620,14 +8360,10 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E128" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr"/>
       <c r="F128" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdditionalTopUpTax/Art4.1.5</t>
@@ -8657,14 +8393,10 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E129" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr"/>
       <c r="F129" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdditionalTopUpTax/Art4.1.5/AdjustedCoveredTax</t>
@@ -8690,14 +8422,10 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E130" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr"/>
       <c r="F130" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdditionalTopUpTax/Art4.1.5/GlobeLoss</t>
@@ -8727,14 +8455,10 @@
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E131" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr"/>
       <c r="F131" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdditionalTopUpTax/Art4.1.5/ExpectedAdjustedCoveredTax</t>
@@ -8764,14 +8488,10 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E132" s="2" t="inlineStr">
-        <is>
-          <t>Ja (fyres aldrig)</t>
-        </is>
-      </c>
+          <t>Slået fra (2026-guidance)</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr"/>
       <c r="F132" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdditionalTopUpTax/Art4.1.5/AdditionalTopUpTax</t>
@@ -8801,14 +8521,10 @@
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E133" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr"/>
       <c r="F133" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdditionalTopUpTax/NONArt4.1.5/Year</t>
@@ -8838,14 +8554,10 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E134" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr"/>
       <c r="F134" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdditionalTopUpTax/NONArt4.1.5/Year</t>
@@ -8875,14 +8587,10 @@
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E135" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr"/>
       <c r="F135" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdditionalTopUpTax/NONArt4.1.5/Year</t>
@@ -8912,14 +8620,10 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E136" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr"/>
       <c r="F136" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/OverallComputation/AdditionalTopUpTax/NONArt4.1.5/AdditionalTopUpTax</t>
@@ -8949,14 +8653,10 @@
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E137" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr"/>
       <c r="F137" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/LowTaxJurisdiction/LTCE/IIR/ParentEntity/InclusionRatio</t>
@@ -8986,14 +8686,10 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E138" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr"/>
       <c r="F138" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/LowTaxJurisdiction/LTCE/IIR/ParentEntity/TopUpTaxShare</t>
@@ -9023,14 +8719,10 @@
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E139" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr"/>
       <c r="F139" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/UTPRAttribution/Attribution/UTPRTopUpTaxAttributed</t>
@@ -9060,14 +8752,10 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E140" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr"/>
       <c r="F140" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/UTPRAttribution</t>
@@ -9097,14 +8785,10 @@
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E141" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr"/>
       <c r="F141" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/UTPRAttribution/Attribution/Employees</t>
@@ -9134,14 +8818,10 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E142" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr"/>
       <c r="F142" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/UTPRAttribution/Attribution/TangibleAssetValue</t>
@@ -9171,14 +8851,10 @@
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E143" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr"/>
       <c r="F143" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/UTPRAttribution/Attribution/UTPRPercentage</t>
@@ -9208,14 +8884,10 @@
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E144" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr"/>
       <c r="F144" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/UTPRAttribution/Attribution/UTPRTopUpTaxCarriedForward</t>
@@ -9241,14 +8913,10 @@
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E145" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr"/>
       <c r="F145" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/UTPRAttribution/Attribution/UTPRTopUpTaxCarriedForward</t>
@@ -9278,14 +8946,10 @@
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E146" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr"/>
       <c r="F146" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedFANIL/Adjustment/CrossBorderAdjustments/OtherTIN</t>
@@ -9315,14 +8979,10 @@
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E147" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr"/>
       <c r="F147" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedFANIL/Total/Adjustment/CrossBorderAdjustments</t>
@@ -9352,14 +9012,10 @@
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E148" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr"/>
       <c r="F148" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedFANIL/Adjustment/UPEAdjustments/IdentificationOfOwners/IndOwners/TaxRateGLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedFANIL/Adjustment/UPEAdjustments/IdentificationOfOwners/EntityOwner/TaxRate</t>
@@ -9389,14 +9045,10 @@
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E149" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr"/>
       <c r="F149" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedFANIL/Adjustment/UPEAdjustments/IdentificationOfOwners/IndOwners</t>
@@ -9426,14 +9078,10 @@
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E150" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr"/>
       <c r="F150" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedFANIL/Adjustment/UPEAdjustments/IdentificationOfOwners/IndOwners</t>
@@ -9463,14 +9111,10 @@
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E151" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr"/>
       <c r="F151" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedFANIL/Adjustment/UPEAdjustments/IdentificationOfOwners/EntityOwner/ExTypeOfEntity</t>
@@ -9500,14 +9144,10 @@
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E152" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr"/>
       <c r="F152" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedFANIL/Adjustment/UPEAdjustments/IdentificationOfOwners/EntityOwner/ExTypeOfEntity</t>
@@ -9537,14 +9177,10 @@
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E153" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr"/>
       <c r="F153" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedFANIL/Adjustment/UPEAdjustments/IdentificationOfOwners/EntityOwner/ExTypeOfEntity</t>
@@ -9574,14 +9210,10 @@
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E154" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr"/>
       <c r="F154" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/NetGlobeIncome/Adjustments/Amount</t>
@@ -9607,14 +9239,10 @@
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E155" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr"/>
       <c r="F155" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLoBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedFANIL/Adjustment/UPEAdjustments</t>
@@ -9644,14 +9272,10 @@
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E156" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr"/>
       <c r="F156" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/NetGlobeIncome/IntShippingIncome</t>
@@ -9681,14 +9305,10 @@
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E157" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr"/>
       <c r="F157" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/Elections/Art7.6</t>
@@ -9718,14 +9338,10 @@
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E158" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr"/>
       <c r="F158" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedCoveredTax/Adjustments/Amount</t>
@@ -9751,12 +9367,12 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Dækket af ækvivalent regel</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Samme semantik håndhæves allerede af regel 70059.</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
@@ -9784,14 +9400,10 @@
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E160" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr"/>
       <c r="F160" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedCoveredTax/DeferTaxAdjustAmt/Total</t>
@@ -9821,12 +9433,12 @@
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Dækket af ækvivalent regel</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
+          <t>Samme semantik håndhæves allerede af regel 70059.</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
@@ -9854,14 +9466,10 @@
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>Nej</t>
-        </is>
-      </c>
-      <c r="E162" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Kandidat (kan kodes)</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr"/>
       <c r="F162" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedCoveredTax/DeferTaxAdjustAmt/Adjustment/Amount</t>
@@ -9887,14 +9495,10 @@
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E163" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr"/>
       <c r="F163" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedIncomeTax/CrossAllocation/Additions</t>
@@ -9920,14 +9524,10 @@
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="E164" s="2" t="inlineStr">
-        <is>
-          <t>Nej</t>
-        </is>
-      </c>
+          <t>Eksekverbar</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr"/>
       <c r="F164" s="2" t="inlineStr">
         <is>
           <t>GLOBEBody/JurisdictionSection/GLOBETax/ETR/ETRStatus/ETRComputation/CEComputation/AdjustedIncomeTax/CrossAllocation/Reductions</t>
@@ -9941,7 +9541,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10098,7 +9698,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Regelkatalog 0.18.0: 92/163 (CEComputation-conditionals + TIN-ulighed) + pakke regenereret
</commit_message>
<xml_diff>
--- a/docs/Pillar2-Validator_Regel-sporbarhedsmatrix.xlsx
+++ b/docs/Pillar2-Validator_Regel-sporbarhedsmatrix.xlsx
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -593,7 +593,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>64%</t>
+          <t>68%</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1970,7 +1970,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>70029</t>
+          <t>70027</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1980,17 +1980,17 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>conditional_ref</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Ownership-TIN (GIR801) skal matche en rapporteret enheds-TIN</t>
+          <t>GlobeStatus GIR318 kræver 0% ejerskab, NOTIN-TIN og GIR806</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70029</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70027</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2012,7 +2012,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>70030</t>
+          <t>70029</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2027,12 +2027,12 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Ownership-TIN (GIR802-804) skal matche en rapporteret enheds-TIN</t>
+          <t>Ownership-TIN (GIR801) skal matche en rapporteret enheds-TIN</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70030</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70029</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2054,7 +2054,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>70032</t>
+          <t>70030</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2064,17 +2064,17 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>conditional_ref</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>QIIR kræver CE-Rules GIR201 eller GIR202</t>
+          <t>Ownership-TIN (GIR802-804) skal matche en rapporteret enheds-TIN</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70032</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70030</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2096,7 +2096,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>70038</t>
+          <t>70032</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2111,12 +2111,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Transitional CbCR SafeHarbour udløber efter 30/06/2028</t>
+          <t>QIIR kræver CE-Rules GIR201 eller GIR202</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70038</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70032</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2138,7 +2138,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>70039</t>
+          <t>70038</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2153,12 +2153,12 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>UTPR SafeHarbour (GIR1206) udløber efter 31/12/2026</t>
+          <t>Transitional CbCR SafeHarbour udløber efter 30/06/2028</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70039</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70038</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2180,7 +2180,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>70044</t>
+          <t>70039</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2195,12 +2195,12 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>ETRStatus skal indeholde ETRException eller ETRComputation</t>
+          <t>UTPR SafeHarbour (GIR1206) udløber efter 31/12/2026</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70044</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70039</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2222,7 +2222,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>70045</t>
+          <t>70044</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2237,12 +2237,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1203-1205 kræver TransitionalCbCRSafeHarbour</t>
+          <t>ETRStatus skal indeholde ETRException eller ETRComputation</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70045</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70044</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2264,7 +2264,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>70047</t>
+          <t>70045</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2279,12 +2279,12 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1203 kræver Revenue</t>
+          <t>SafeHarbour GIR1203-1205 kræver TransitionalCbCRSafeHarbour</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70047</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70045</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>70048</t>
+          <t>70047</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2321,12 +2321,12 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1204 kræver IncomeTax</t>
+          <t>SafeHarbour GIR1203 kræver Revenue</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70048</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70047</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2348,7 +2348,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>70049</t>
+          <t>70048</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2363,12 +2363,12 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1206 kræver UTPRSafeHarbour</t>
+          <t>SafeHarbour GIR1204 kræver IncomeTax</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70049</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70048</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2390,7 +2390,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>70051</t>
+          <t>70049</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2405,12 +2405,12 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1208 kræver AggregateSimplified</t>
+          <t>SafeHarbour GIR1206 kræver UTPRSafeHarbour</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70051</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70049</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2432,7 +2432,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>70055</t>
+          <t>70051</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2442,17 +2442,17 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>OutstandingBalance-beregning</t>
+          <t>SafeHarbour GIR1208 kræver AggregateSimplified</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70055</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70051</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2474,7 +2474,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>70059</t>
+          <t>70055</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2484,17 +2484,17 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>unique_in</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem-kode kun én gang pr. ETR</t>
+          <t>OutstandingBalance-beregning</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70059</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70055</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2516,7 +2516,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>70060</t>
+          <t>70058</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2526,17 +2526,17 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>not_equal</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem GIR2025 kræver IntShippingIncome</t>
+          <t>InvestmentEntityTIN må ikke matche CEComputation-TIN</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70060</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70058</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2558,7 +2558,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>70062</t>
+          <t>70059</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2568,17 +2568,17 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>unique_in</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem GIR2720 udelukker negativ AdjustedCoveredTax</t>
+          <t>AdjustmentItem-kode kun én gang pr. ETR</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70062</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70059</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2600,7 +2600,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>70064</t>
+          <t>70060</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2610,17 +2610,17 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>DeferTaxAsset/Total-beregning</t>
+          <t>AdjustmentItem GIR2025 kræver IntShippingIncome</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70064</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70060</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2642,7 +2642,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>70065</t>
+          <t>70062</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2652,17 +2652,17 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>CoveredTaxRefund/Total-beregning</t>
+          <t>AdjustmentItem GIR2720 udelukker negativ AdjustedCoveredTax</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70065</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70062</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2684,7 +2684,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>70066</t>
+          <t>70064</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>DeferTaxAsset-år må ikke ligge efter periodens start</t>
+          <t>DeferTaxAsset/Total-beregning</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70066</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70064</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2726,7 +2726,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>70067</t>
+          <t>70065</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2736,17 +2736,17 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>unique_in</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>AmountAttributed-år skal være unikke</t>
+          <t>CoveredTaxRefund/Total-beregning</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70067</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70065</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2768,7 +2768,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>70068</t>
+          <t>70066</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2783,12 +2783,12 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>CoveredTaxRefund-år må ikke ligge efter periodens start</t>
+          <t>DeferTaxAsset-år må ikke ligge efter periodens start</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70068</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70066</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2810,7 +2810,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>70070</t>
+          <t>70067</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2820,17 +2820,17 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>unique_in</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Recapture-år må ikke ligge efter periodens slut</t>
+          <t>AmountAttributed-år skal være unikke</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70070</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70067</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2852,7 +2852,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>70071</t>
+          <t>70068</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2862,17 +2862,17 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Recapture-år må ikke være 4+ år før periodens slut</t>
+          <t>CoveredTaxRefund-år må ikke ligge efter periodens start</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70071</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70068</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2894,7 +2894,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>70072</t>
+          <t>70070</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2904,17 +2904,17 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>EndAmount-beregning (DDT-recapture)</t>
+          <t>Recapture-år må ikke ligge efter periodens slut</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70072</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70070</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -2936,7 +2936,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>70073</t>
+          <t>70071</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2946,17 +2946,17 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>value_range</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>EndAmount må ikke være negativ</t>
+          <t>Recapture-år må ikke være 4+ år før periodens slut</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70073</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70071</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2978,7 +2978,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>70074</t>
+          <t>70072</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2993,12 +2993,12 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>TotalDDT-beregning</t>
+          <t>EndAmount-beregning (DDT-recapture)</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70074</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70072</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -3020,7 +3020,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>70076</t>
+          <t>70073</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -3030,17 +3030,17 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>value_range</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>TransBlendCFC/Total-beregning</t>
+          <t>EndAmount må ikke være negativ</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70076</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70073</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -3062,7 +3062,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>70077</t>
+          <t>70074</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -3077,12 +3077,12 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>DeferTaxAdjustAmt/Total-beregning (Recast)</t>
+          <t>TotalDDT-beregning</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70077</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70074</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -3104,7 +3104,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>70078</t>
+          <t>70076</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -3119,12 +3119,12 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>BefRecastAdjust-beregning</t>
+          <t>TransBlendCFC/Total-beregning</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70078</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70076</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>70079</t>
+          <t>70077</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -3161,12 +3161,12 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>PreRecast-beregning</t>
+          <t>DeferTaxAdjustAmt/Total-beregning (Recast)</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70079</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70077</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -3188,7 +3188,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>70082</t>
+          <t>70078</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3198,17 +3198,17 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>DeferredTaxAssets kræver Start eller Recast = 0</t>
+          <t>BefRecastAdjust-beregning</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70082</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70078</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -3230,7 +3230,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>70083</t>
+          <t>70079</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3245,12 +3245,12 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>ExcessNegTaxExpense/Remaining-beregning</t>
+          <t>PreRecast-beregning</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70083</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70079</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -3272,7 +3272,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>70086</t>
+          <t>70082</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3282,17 +3282,17 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>ExcessProfits-beregning</t>
+          <t>DeferredTaxAssets kræver Start eller Recast = 0</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70086</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70082</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -3314,7 +3314,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>70087</t>
+          <t>70083</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -3329,12 +3329,12 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>SubstanceExclusion/Total-beregning</t>
+          <t>ExcessNegTaxExpense/Remaining-beregning</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70087</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70083</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -3356,7 +3356,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>70088</t>
+          <t>70086</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3366,17 +3366,17 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Negativ NetGlobeIncome kræver Art4.1.5</t>
+          <t>ExcessProfits-beregning</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70088</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70086</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -3398,7 +3398,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>70090</t>
+          <t>70087</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3413,12 +3413,12 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>GlobeLoss skal svare til NetGlobeIncome/Total</t>
+          <t>SubstanceExclusion/Total-beregning</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70090</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70087</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -3440,7 +3440,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>70091</t>
+          <t>70088</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3450,17 +3450,17 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>ExpectedAdjustedCoveredTax = GlobeLoss × 15%</t>
+          <t>Negativ NetGlobeIncome kræver Art4.1.5</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70091</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70088</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -3482,7 +3482,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>70093</t>
+          <t>70090</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3492,17 +3492,17 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>NONArt4.1.5-år må ikke overstige periodens slut</t>
+          <t>GlobeLoss skal svare til NetGlobeIncome/Total</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70093</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70090</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -3524,7 +3524,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>70094</t>
+          <t>70091</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3534,17 +3534,17 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Articles GIR2605 kræver år mindst 4 år før periodens slut</t>
+          <t>ExpectedAdjustedCoveredTax = GlobeLoss × 15%</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70094</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70091</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -3566,7 +3566,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>70095</t>
+          <t>70093</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -3576,17 +3576,17 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Articles GIR2602 kræver det femte år før periodens slut</t>
+          <t>NONArt4.1.5-år må ikke overstige periodens slut</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70095</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70093</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -3608,7 +3608,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>70097</t>
+          <t>70094</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3618,17 +3618,17 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>InclusionRatio-beregning</t>
+          <t>Articles GIR2605 kræver år mindst 4 år før periodens slut</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70097</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70094</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -3650,7 +3650,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>70098</t>
+          <t>70095</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3660,17 +3660,17 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>TopUpTaxShare = TopUpTax × InclusionRatio</t>
+          <t>Articles GIR2602 kræver det femte år før periodens slut</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70098</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70095</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -3692,7 +3692,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>70101</t>
+          <t>70097</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3702,17 +3702,17 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Employees kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
+          <t>InclusionRatio-beregning</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70101</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70097</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -3734,7 +3734,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>70102</t>
+          <t>70098</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -3744,17 +3744,17 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>TangibleAssetValue kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
+          <t>TopUpTaxShare = TopUpTax × InclusionRatio</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70102</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70098</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -3776,7 +3776,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>70103</t>
+          <t>70101</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -3791,12 +3791,12 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>UTPRPercentage skal være 0 når carryforward &gt; 0</t>
+          <t>Employees kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70103</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70101</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -3818,7 +3818,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>70104</t>
+          <t>70102</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -3828,17 +3828,17 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>value_range</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>UTPRTopUpTaxCarriedForward må ikke være negativ</t>
+          <t>TangibleAssetValue kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70104</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70102</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -3860,7 +3860,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>70105</t>
+          <t>70103</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3870,17 +3870,17 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>UTPRTopUpTaxCarriedForward-beregning</t>
+          <t>UTPRPercentage skal være 0 når carryforward &gt; 0</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70105</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70103</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -3902,7 +3902,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>70107</t>
+          <t>70104</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -3912,17 +3912,17 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>value_range</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Exception=TRUE udelukker CrossBorderAdjustments</t>
+          <t>UTPRTopUpTaxCarriedForward må ikke være negativ</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70107</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70104</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -3944,7 +3944,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>70108</t>
+          <t>70105</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -3954,17 +3954,17 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Basis kræver TaxRate</t>
+          <t>UTPRTopUpTaxCarriedForward-beregning</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70108</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70105</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -3986,7 +3986,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>70109</t>
+          <t>70106</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -3996,17 +3996,17 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>not_equal</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1907 kræver IndOwners/ResCountryCode</t>
+          <t>OtherTIN må ikke matche CEComputation-TIN</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70109</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70106</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -4028,7 +4028,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>70110</t>
+          <t>70107</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -4043,12 +4043,12 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1903/1908 kræver IndOwners</t>
+          <t>Exception=TRUE udelukker CrossBorderAdjustments</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70110</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70107</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -4070,7 +4070,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>70111</t>
+          <t>70108</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -4085,12 +4085,12 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1904/1909 kræver EntityOwner/ExTypeOfEntity</t>
+          <t>Basis kræver TaxRate</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70111</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70108</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -4112,7 +4112,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>70112</t>
+          <t>70109</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -4127,12 +4127,12 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1904 udelukker ExTypeOfEntity GIR2805</t>
+          <t>Basis GIR1907 kræver IndOwners/ResCountryCode</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70112</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70109</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -4154,7 +4154,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>70113</t>
+          <t>70110</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -4169,12 +4169,12 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1909 udelukker ExTypeOfEntity GIR2804</t>
+          <t>Basis GIR1903/1908 kræver IndOwners</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70113</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70110</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -4196,7 +4196,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>70115</t>
+          <t>70111</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4211,12 +4211,12 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem GIR2022/2023 kræver UPEAdjustments</t>
+          <t>Basis GIR1904/1909 kræver EntityOwner/ExTypeOfEntity</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70115</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70111</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -4238,7 +4238,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>70123</t>
+          <t>70112</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -4248,17 +4248,17 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>value_range</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Additions må ikke være negativ</t>
+          <t>Basis GIR1904 udelukker ExTypeOfEntity GIR2805</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70123</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70112</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -4280,40 +4280,250 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
+          <t>70113</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Basis GIR1909 udelukker ExTypeOfEntity GIR2804</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70113</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>70115</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>AdjustmentItem GIR2022/2023 kræver UPEAdjustments</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70115</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>70116</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>AdjustmentItem GIR2025 kræver IntShippingIncome (CEComputation)</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70116</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>70117</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>AdjustmentItem GIR2024 kræver Art7.6 (CEComputation)</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70117</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>70123</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>value_range</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Additions må ikke være negativ</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70123</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
           <t>70124</t>
         </is>
       </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="C88" s="2" t="inlineStr">
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
         <is>
           <t>value_range</t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr">
+      <c r="D93" s="2" t="inlineStr">
         <is>
           <t>CrossAllocation/Reductions må ikke være positiv</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr">
+      <c r="E93" s="2" t="inlineStr">
         <is>
           <t>OECD Status Message User Guide Part 4 — regel 70124</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr">
+      <c r="F93" s="2" t="inlineStr">
         <is>
           <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
         </is>
       </c>
-      <c r="G88" s="2" t="inlineStr">
+      <c r="G93" s="2" t="inlineStr">
         <is>
           <t>Ja — auto-scenarie (bestået)</t>
         </is>
       </c>
-      <c r="H88" s="2" t="inlineStr">
+      <c r="H93" s="2" t="inlineStr">
         <is>
           <t>Væsentlig (High)</t>
         </is>
@@ -6379,7 +6589,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Kandidat (kan kodes)</t>
+          <t>Eksekverbar</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr"/>
@@ -7386,7 +7596,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Kandidat (kan kodes)</t>
+          <t>Eksekverbar</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr"/>
@@ -8946,7 +9156,7 @@
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>Kandidat (kan kodes)</t>
+          <t>Eksekverbar</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr"/>
@@ -9272,7 +9482,7 @@
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>Kandidat (kan kodes)</t>
+          <t>Eksekverbar</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr"/>
@@ -9305,7 +9515,7 @@
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>Kandidat (kan kodes)</t>
+          <t>Eksekverbar</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Regelkatalog 0.19.0: 97/163 (kryds-sektion-conditionals) + fixtur-tests peger paa golden + pakke regenereret
</commit_message>
<xml_diff>
--- a/docs/Pillar2-Validator_Regel-sporbarhedsmatrix.xlsx
+++ b/docs/Pillar2-Validator_Regel-sporbarhedsmatrix.xlsx
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -593,7 +593,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>68%</t>
+          <t>71%</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -878,7 +878,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>60020</t>
+          <t>60016</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -888,17 +888,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Periodens startdato må ikke ligge efter slutdato</t>
+          <t>FilingInfo OECD0 → GeneralSection må ikke være OECD1</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 60020</t>
+          <t>OECD Status Message User Guide Part 4 — regel 60016</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -920,7 +920,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>60021</t>
+          <t>60017</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Periodens slutdato må ikke ligge efter rapporteringsperioden</t>
+          <t>FilingInfo OECD1 kræver GeneralSection</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 60021</t>
+          <t>OECD Status Message User Guide Part 4 — regel 60017</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -962,7 +962,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>60023</t>
+          <t>60020</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -977,12 +977,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>FilingCE's land skal matche afsenderlandet</t>
+          <t>Periodens startdato må ikke ligge efter slutdato</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 60023</t>
+          <t>OECD Status Message User Guide Part 4 — regel 60020</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1004,7 +1004,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>60027</t>
+          <t>60021</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1014,17 +1014,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>IIR ParentEntity TopUpTax-beregning</t>
+          <t>Periodens slutdato må ikke ligge efter rapporteringsperioden</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 60027</t>
+          <t>OECD Status Message User Guide Part 4 — regel 60021</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1046,7 +1046,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>70015</t>
+          <t>60023</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1056,17 +1056,17 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>GIR308 kræver en tilsvarende GIR307-enhed</t>
+          <t>FilingCE's land skal matche afsenderlandet</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70015</t>
+          <t>OECD Status Message User Guide Part 4 — regel 60023</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1088,7 +1088,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>70019</t>
+          <t>60024</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1103,12 +1103,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>GIR305 kræver en tilsvarende GIR306-enhed</t>
+          <t>Summary-indhold kræver JurWithTaxingRights/JurisdictionName</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70019</t>
+          <t>OECD Status Message User Guide Part 4 — regel 60024</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1130,7 +1130,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>70041</t>
+          <t>60027</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1140,17 +1140,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>CFSofUPE GIR502/504 udelukker SafeHarbour GIR1207-1209</t>
+          <t>IIR ParentEntity TopUpTax-beregning</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70041</t>
+          <t>OECD Status Message User Guide Part 4 — regel 60027</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1172,27 +1172,27 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>60028</t>
+          <t>70015</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>record</t>
+          <t>file</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>AdjustedFANIL/Total-beregning</t>
+          <t>GIR308 kræver en tilsvarende GIR307-enhed</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 60028</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70015</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1214,12 +1214,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>70001</t>
+          <t>70019</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>record</t>
+          <t>file</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1229,12 +1229,12 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>NOTIN-TIN skal udfyldes korrekt</t>
+          <t>GIR305 kræver en tilsvarende GIR306-enhed</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70001</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70019</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1256,12 +1256,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>70002</t>
+          <t>70041</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>record</t>
+          <t>file</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>TIN='NOTIN' kræver TypeOfTIN=GIR3004</t>
+          <t>CFSofUPE GIR502/504 udelukker SafeHarbour GIR1207-1209</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70002</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70041</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1298,7 +1298,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>70003</t>
+          <t>60028</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1308,17 +1308,17 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Unknown-TIN skal udfyldes korrekt</t>
+          <t>AdjustedFANIL/Total-beregning</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70003</t>
+          <t>OECD Status Message User Guide Part 4 — regel 60028</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1340,7 +1340,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>70005</t>
+          <t>70001</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>issuedBy kræves for almindelige TIN</t>
+          <t>NOTIN-TIN skal udfyldes korrekt</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70005</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70001</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1382,7 +1382,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>70009</t>
+          <t>70002</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1397,12 +1397,12 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Ugyldig GlobeStatus for UPE</t>
+          <t>TIN='NOTIN' kræver TypeOfTIN=GIR3004</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70009</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70002</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1424,7 +1424,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>70010</t>
+          <t>70003</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1434,17 +1434,17 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>cardinality</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>UPE må kun have ét ResCountryCode</t>
+          <t>Unknown-TIN skal udfyldes korrekt</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70010</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70003</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1466,7 +1466,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>70011</t>
+          <t>70005</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1476,17 +1476,17 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>cardinality</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>CE må kun have ét ResCountryCode</t>
+          <t>issuedBy kræves for almindelige TIN</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70011</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70005</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1508,7 +1508,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>70013</t>
+          <t>70009</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1523,12 +1523,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>GIR313 og GIR314 udelukker hinanden (samme CE)</t>
+          <t>Ugyldig GlobeStatus for UPE</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70013</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70009</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1550,7 +1550,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>70014</t>
+          <t>70010</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1560,17 +1560,17 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>cardinality</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>GIR307 og GIR308 udelukker hinanden (samme CE)</t>
+          <t>UPE må kun have ét ResCountryCode</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70014</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70010</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1592,7 +1592,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>70016</t>
+          <t>70011</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1602,17 +1602,17 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>cardinality</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>GlobeStatus GIR307 kræver GIR309</t>
+          <t>CE må kun have ét ResCountryCode</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70016</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70011</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1634,7 +1634,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>70017</t>
+          <t>70013</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1649,12 +1649,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>GlobeStatus GIR308 kræver GIR309</t>
+          <t>GIR313 og GIR314 udelukker hinanden (samme CE)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70017</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70013</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1676,7 +1676,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>70018</t>
+          <t>70014</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1691,12 +1691,12 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>GIR305 og GIR306 udelukker hinanden (samme CE)</t>
+          <t>GIR307 og GIR308 udelukker hinanden (samme CE)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70018</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70014</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1718,7 +1718,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>70021</t>
+          <t>70016</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1733,12 +1733,12 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>GlobeStatus GIR316/318 kræver OwnershipChange</t>
+          <t>GlobeStatus GIR307 kræver GIR309</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70021</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70016</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1760,7 +1760,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>70022</t>
+          <t>70017</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1770,17 +1770,17 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>ChangeDate må ikke ligge før periodens start</t>
+          <t>GlobeStatus GIR308 kræver GIR309</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70022</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70017</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1802,7 +1802,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>70023</t>
+          <t>70018</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1812,17 +1812,17 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>ChangeDate må ikke ligge efter periodens slutning</t>
+          <t>GIR305 og GIR306 udelukker hinanden (samme CE)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70023</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70018</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1844,7 +1844,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>70024</t>
+          <t>70021</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1859,12 +1859,12 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>PreOwnership må ikke udfyldes ved PreGlobeStatus GIR719</t>
+          <t>GlobeStatus GIR316/318 kræver OwnershipChange</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70024</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70021</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1886,7 +1886,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>70025</t>
+          <t>70022</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1896,17 +1896,17 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Nominee-PreOwnership kræver NOTIN-TIN</t>
+          <t>ChangeDate må ikke ligge før periodens start</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70025</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70022</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1928,7 +1928,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>70026</t>
+          <t>70023</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1938,17 +1938,17 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>GlobeStatus GIR305 kræver 100% ejerskab</t>
+          <t>ChangeDate må ikke ligge efter periodens slutning</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70026</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70023</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1970,7 +1970,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>70027</t>
+          <t>70024</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1985,12 +1985,12 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>GlobeStatus GIR318 kræver 0% ejerskab, NOTIN-TIN og GIR806</t>
+          <t>PreOwnership må ikke udfyldes ved PreGlobeStatus GIR719</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70027</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70024</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2012,7 +2012,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>70029</t>
+          <t>70025</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2022,17 +2022,17 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>conditional_ref</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Ownership-TIN (GIR801) skal matche en rapporteret enheds-TIN</t>
+          <t>Nominee-PreOwnership kræver NOTIN-TIN</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70029</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70025</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2054,7 +2054,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>70030</t>
+          <t>70026</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2064,17 +2064,17 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>conditional_ref</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Ownership-TIN (GIR802-804) skal matche en rapporteret enheds-TIN</t>
+          <t>GlobeStatus GIR305 kræver 100% ejerskab</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70030</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70026</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2096,7 +2096,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>70032</t>
+          <t>70027</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2111,12 +2111,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>QIIR kræver CE-Rules GIR201 eller GIR202</t>
+          <t>GlobeStatus GIR318 kræver 0% ejerskab, NOTIN-TIN og GIR806</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70032</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70027</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2138,7 +2138,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>70038</t>
+          <t>70029</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2148,17 +2148,17 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>conditional_ref</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Transitional CbCR SafeHarbour udløber efter 30/06/2028</t>
+          <t>Ownership-TIN (GIR801) skal matche en rapporteret enheds-TIN</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70038</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70029</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2180,7 +2180,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>70039</t>
+          <t>70030</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2190,17 +2190,17 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>conditional_ref</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>UTPR SafeHarbour (GIR1206) udløber efter 31/12/2026</t>
+          <t>Ownership-TIN (GIR802-804) skal matche en rapporteret enheds-TIN</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70039</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70030</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2222,7 +2222,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>70044</t>
+          <t>70032</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2237,12 +2237,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>ETRStatus skal indeholde ETRException eller ETRComputation</t>
+          <t>QIIR kræver CE-Rules GIR201 eller GIR202</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70044</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70032</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2264,7 +2264,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>70045</t>
+          <t>70038</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2279,12 +2279,12 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1203-1205 kræver TransitionalCbCRSafeHarbour</t>
+          <t>Transitional CbCR SafeHarbour udløber efter 30/06/2028</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70045</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70038</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>70047</t>
+          <t>70039</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2321,12 +2321,12 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1203 kræver Revenue</t>
+          <t>UTPR SafeHarbour (GIR1206) udløber efter 31/12/2026</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70047</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70039</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2348,7 +2348,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>70048</t>
+          <t>70043</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2363,12 +2363,12 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1204 kræver IncomeTax</t>
+          <t>JurWithTaxingRights + SafeHarbour GIR1202 kræver ETRRange/SBIE/QDMTTut</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70048</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70043</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2390,7 +2390,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>70049</t>
+          <t>70044</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2405,12 +2405,12 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1206 kræver UTPRSafeHarbour</t>
+          <t>ETRStatus skal indeholde ETRException eller ETRComputation</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70049</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70044</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2432,7 +2432,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>70051</t>
+          <t>70045</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2447,12 +2447,12 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>SafeHarbour GIR1208 kræver AggregateSimplified</t>
+          <t>SafeHarbour GIR1203-1205 kræver TransitionalCbCRSafeHarbour</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70051</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70045</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2474,7 +2474,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>70055</t>
+          <t>70046</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2484,17 +2484,17 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>OutstandingBalance-beregning</t>
+          <t>TransitionalCbCRSafeHarbour kræver SubGroup med GIR1607/1608</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70055</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70046</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2516,7 +2516,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>70058</t>
+          <t>70047</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2526,17 +2526,17 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>not_equal</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>InvestmentEntityTIN må ikke matche CEComputation-TIN</t>
+          <t>SafeHarbour GIR1203 kræver Revenue</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70058</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70047</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2558,7 +2558,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>70059</t>
+          <t>70048</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2568,17 +2568,17 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>unique_in</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem-kode kun én gang pr. ETR</t>
+          <t>SafeHarbour GIR1204 kræver IncomeTax</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70059</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70048</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2600,7 +2600,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>70060</t>
+          <t>70049</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2615,12 +2615,12 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem GIR2025 kræver IntShippingIncome</t>
+          <t>SafeHarbour GIR1206 kræver UTPRSafeHarbour</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70060</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70049</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2642,7 +2642,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>70062</t>
+          <t>70051</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2657,12 +2657,12 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem GIR2720 udelukker negativ AdjustedCoveredTax</t>
+          <t>SafeHarbour GIR1208 kræver AggregateSimplified</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70062</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70051</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2684,7 +2684,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>70064</t>
+          <t>70055</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2699,12 +2699,12 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>DeferTaxAsset/Total-beregning</t>
+          <t>OutstandingBalance-beregning</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70064</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70055</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2726,7 +2726,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>70065</t>
+          <t>70058</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2736,17 +2736,17 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>not_equal</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>CoveredTaxRefund/Total-beregning</t>
+          <t>InvestmentEntityTIN må ikke matche CEComputation-TIN</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70065</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70058</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2768,7 +2768,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>70066</t>
+          <t>70059</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2778,17 +2778,17 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>unique_in</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>DeferTaxAsset-år må ikke ligge efter periodens start</t>
+          <t>AdjustmentItem-kode kun én gang pr. ETR</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70066</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70059</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2810,7 +2810,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>70067</t>
+          <t>70060</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2820,17 +2820,17 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>unique_in</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>AmountAttributed-år skal være unikke</t>
+          <t>AdjustmentItem GIR2025 kræver IntShippingIncome</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70067</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70060</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2852,7 +2852,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>70068</t>
+          <t>70062</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2862,17 +2862,17 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>CoveredTaxRefund-år må ikke ligge efter periodens start</t>
+          <t>AdjustmentItem GIR2720 udelukker negativ AdjustedCoveredTax</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70068</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70062</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2894,7 +2894,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>70070</t>
+          <t>70064</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2904,17 +2904,17 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Recapture-år må ikke ligge efter periodens slut</t>
+          <t>DeferTaxAsset/Total-beregning</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70070</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70064</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -2936,7 +2936,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>70071</t>
+          <t>70065</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2946,17 +2946,17 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Recapture-år må ikke være 4+ år før periodens slut</t>
+          <t>CoveredTaxRefund/Total-beregning</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70071</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70065</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2978,7 +2978,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>70072</t>
+          <t>70066</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2988,17 +2988,17 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>EndAmount-beregning (DDT-recapture)</t>
+          <t>DeferTaxAsset-år må ikke ligge efter periodens start</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70072</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70066</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -3020,7 +3020,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>70073</t>
+          <t>70067</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -3030,17 +3030,17 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>value_range</t>
+          <t>unique_in</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>EndAmount må ikke være negativ</t>
+          <t>AmountAttributed-år skal være unikke</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70073</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70067</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -3062,7 +3062,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>70074</t>
+          <t>70068</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -3072,17 +3072,17 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>TotalDDT-beregning</t>
+          <t>CoveredTaxRefund-år må ikke ligge efter periodens start</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70074</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70068</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -3104,7 +3104,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>70076</t>
+          <t>70070</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -3114,17 +3114,17 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>TransBlendCFC/Total-beregning</t>
+          <t>Recapture-år må ikke ligge efter periodens slut</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70076</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70070</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>70077</t>
+          <t>70071</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -3156,17 +3156,17 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>DeferTaxAdjustAmt/Total-beregning (Recast)</t>
+          <t>Recapture-år må ikke være 4+ år før periodens slut</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70077</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70071</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -3188,7 +3188,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>70078</t>
+          <t>70072</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3203,12 +3203,12 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>BefRecastAdjust-beregning</t>
+          <t>EndAmount-beregning (DDT-recapture)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70078</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70072</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -3230,7 +3230,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>70079</t>
+          <t>70073</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3240,17 +3240,17 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>value_range</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>PreRecast-beregning</t>
+          <t>EndAmount må ikke være negativ</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70079</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70073</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -3272,7 +3272,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>70082</t>
+          <t>70074</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3282,17 +3282,17 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>DeferredTaxAssets kræver Start eller Recast = 0</t>
+          <t>TotalDDT-beregning</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70082</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70074</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -3314,7 +3314,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>70083</t>
+          <t>70076</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -3329,12 +3329,12 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>ExcessNegTaxExpense/Remaining-beregning</t>
+          <t>TransBlendCFC/Total-beregning</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70083</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70076</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -3356,7 +3356,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>70086</t>
+          <t>70077</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3371,12 +3371,12 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>ExcessProfits-beregning</t>
+          <t>DeferTaxAdjustAmt/Total-beregning (Recast)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70086</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70077</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -3398,7 +3398,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>70087</t>
+          <t>70078</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3413,12 +3413,12 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>SubstanceExclusion/Total-beregning</t>
+          <t>BefRecastAdjust-beregning</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70087</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70078</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -3440,7 +3440,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>70088</t>
+          <t>70079</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3450,17 +3450,17 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Negativ NetGlobeIncome kræver Art4.1.5</t>
+          <t>PreRecast-beregning</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70088</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70079</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -3482,7 +3482,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>70090</t>
+          <t>70082</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3492,17 +3492,17 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>calculation</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>GlobeLoss skal svare til NetGlobeIncome/Total</t>
+          <t>DeferredTaxAssets kræver Start eller Recast = 0</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70090</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70082</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -3524,7 +3524,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>70091</t>
+          <t>70083</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3539,12 +3539,12 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>ExpectedAdjustedCoveredTax = GlobeLoss × 15%</t>
+          <t>ExcessNegTaxExpense/Remaining-beregning</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70091</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70083</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -3566,7 +3566,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>70093</t>
+          <t>70086</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -3576,17 +3576,17 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>NONArt4.1.5-år må ikke overstige periodens slut</t>
+          <t>ExcessProfits-beregning</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70093</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70086</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -3608,7 +3608,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>70094</t>
+          <t>70087</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3618,17 +3618,17 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Articles GIR2605 kræver år mindst 4 år før periodens slut</t>
+          <t>SubstanceExclusion/Total-beregning</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70094</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70087</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -3650,7 +3650,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>70095</t>
+          <t>70088</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3665,12 +3665,12 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Articles GIR2602 kræver det femte år før periodens slut</t>
+          <t>Negativ NetGlobeIncome kræver Art4.1.5</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70095</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70088</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -3692,7 +3692,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>70097</t>
+          <t>70090</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3707,12 +3707,12 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>InclusionRatio-beregning</t>
+          <t>GlobeLoss skal svare til NetGlobeIncome/Total</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70097</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70090</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -3734,7 +3734,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>70098</t>
+          <t>70091</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -3749,12 +3749,12 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>TopUpTaxShare = TopUpTax × InclusionRatio</t>
+          <t>ExpectedAdjustedCoveredTax = GlobeLoss × 15%</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70098</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70091</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -3776,7 +3776,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>70101</t>
+          <t>70093</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -3786,17 +3786,17 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Employees kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
+          <t>NONArt4.1.5-år må ikke overstige periodens slut</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70101</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70093</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -3818,7 +3818,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>70102</t>
+          <t>70094</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -3833,12 +3833,12 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>TangibleAssetValue kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
+          <t>Articles GIR2605 kræver år mindst 4 år før periodens slut</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70102</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70094</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -3860,7 +3860,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>70103</t>
+          <t>70095</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3875,12 +3875,12 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>UTPRPercentage skal være 0 når carryforward &gt; 0</t>
+          <t>Articles GIR2602 kræver det femte år før periodens slut</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70103</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70095</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -3902,7 +3902,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>70104</t>
+          <t>70097</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -3912,17 +3912,17 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>value_range</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>UTPRTopUpTaxCarriedForward må ikke være negativ</t>
+          <t>InclusionRatio-beregning</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70104</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70097</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -3944,7 +3944,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>70105</t>
+          <t>70098</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -3959,12 +3959,12 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>UTPRTopUpTaxCarriedForward-beregning</t>
+          <t>TopUpTaxShare = TopUpTax × InclusionRatio</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70105</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70098</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -3986,7 +3986,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>70106</t>
+          <t>70101</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -3996,17 +3996,17 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>not_equal</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>OtherTIN må ikke matche CEComputation-TIN</t>
+          <t>Employees kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70106</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70101</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -4028,7 +4028,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>70107</t>
+          <t>70102</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -4043,12 +4043,12 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Exception=TRUE udelukker CrossBorderAdjustments</t>
+          <t>TangibleAssetValue kræves når UTPRTopUpTaxCarryForward ≠ 0</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70107</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70102</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -4070,7 +4070,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>70108</t>
+          <t>70103</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -4085,12 +4085,12 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Basis kræver TaxRate</t>
+          <t>UTPRPercentage skal være 0 når carryforward &gt; 0</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70108</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70103</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -4112,7 +4112,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>70109</t>
+          <t>70104</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -4122,17 +4122,17 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>value_range</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1907 kræver IndOwners/ResCountryCode</t>
+          <t>UTPRTopUpTaxCarriedForward må ikke være negativ</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70109</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70104</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -4154,7 +4154,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>70110</t>
+          <t>70105</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -4164,17 +4164,17 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>calculation</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1903/1908 kræver IndOwners</t>
+          <t>UTPRTopUpTaxCarriedForward-beregning</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70110</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70105</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -4196,7 +4196,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>70111</t>
+          <t>70106</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4206,17 +4206,17 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>not_equal</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1904/1909 kræver EntityOwner/ExTypeOfEntity</t>
+          <t>OtherTIN må ikke matche CEComputation-TIN</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70111</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70106</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -4238,7 +4238,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>70112</t>
+          <t>70107</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -4253,12 +4253,12 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1904 udelukker ExTypeOfEntity GIR2805</t>
+          <t>Exception=TRUE udelukker CrossBorderAdjustments</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70112</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70107</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -4280,7 +4280,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>70113</t>
+          <t>70108</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4295,12 +4295,12 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Basis GIR1909 udelukker ExTypeOfEntity GIR2804</t>
+          <t>Basis kræver TaxRate</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70113</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70108</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -4322,7 +4322,7 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>70115</t>
+          <t>70109</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -4337,12 +4337,12 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem GIR2022/2023 kræver UPEAdjustments</t>
+          <t>Basis GIR1907 kræver IndOwners/ResCountryCode</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70115</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70109</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
@@ -4364,7 +4364,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>70116</t>
+          <t>70110</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4379,12 +4379,12 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem GIR2025 kræver IntShippingIncome (CEComputation)</t>
+          <t>Basis GIR1903/1908 kræver IndOwners</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70116</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70110</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -4406,7 +4406,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>70117</t>
+          <t>70111</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -4421,12 +4421,12 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>AdjustmentItem GIR2024 kræver Art7.6 (CEComputation)</t>
+          <t>Basis GIR1904/1909 kræver EntityOwner/ExTypeOfEntity</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70117</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70111</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
@@ -4448,7 +4448,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>70123</t>
+          <t>70112</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4458,17 +4458,17 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>value_range</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Additions må ikke være negativ</t>
+          <t>Basis GIR1904 udelukker ExTypeOfEntity GIR2805</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>OECD Status Message User Guide Part 4 — regel 70123</t>
+          <t>OECD Status Message User Guide Part 4 — regel 70112</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -4490,40 +4490,250 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
+          <t>70113</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Basis GIR1909 udelukker ExTypeOfEntity GIR2804</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70113</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>70115</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>AdjustmentItem GIR2022/2023 kræver UPEAdjustments</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70115</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>70116</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>AdjustmentItem GIR2025 kræver IntShippingIncome (CEComputation)</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70116</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>70117</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>AdjustmentItem GIR2024 kræver Art7.6 (CEComputation)</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70117</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>70123</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>value_range</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Additions må ikke være negativ</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>OECD Status Message User Guide Part 4 — regel 70123</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Ja — auto-scenarie (bestået)</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Væsentlig (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
           <t>70124</t>
         </is>
       </c>
-      <c r="B93" s="2" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="C93" s="2" t="inlineStr">
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
         <is>
           <t>value_range</t>
         </is>
       </c>
-      <c r="D93" s="2" t="inlineStr">
+      <c r="D98" s="2" t="inlineStr">
         <is>
           <t>CrossAllocation/Reductions må ikke være positiv</t>
         </is>
       </c>
-      <c r="E93" s="2" t="inlineStr">
+      <c r="E98" s="2" t="inlineStr">
         <is>
           <t>OECD Status Message User Guide Part 4 — regel 70124</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr">
+      <c r="F98" s="2" t="inlineStr">
         <is>
           <t>validator/rules/oecd_rules.py (datadrevet motor)</t>
         </is>
       </c>
-      <c r="G93" s="2" t="inlineStr">
+      <c r="G98" s="2" t="inlineStr">
         <is>
           <t>Ja — auto-scenarie (bestået)</t>
         </is>
       </c>
-      <c r="H93" s="2" t="inlineStr">
+      <c r="H98" s="2" t="inlineStr">
         <is>
           <t>Væsentlig (High)</t>
         </is>
@@ -5390,7 +5600,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Kandidat (kan kodes)</t>
+          <t>Eksekverbar</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
@@ -5419,7 +5629,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Kandidat (kan kodes)</t>
+          <t>Eksekverbar</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
@@ -5638,7 +5848,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Kandidat (kan kodes)</t>
+          <t>Eksekverbar</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr"/>
@@ -7113,7 +7323,7 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Kandidat (kan kodes)</t>
+          <t>Eksekverbar</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr"/>
@@ -7208,7 +7418,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Kandidat (kan kodes)</t>
+          <t>Eksekverbar</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr"/>

</xml_diff>